<commit_message>
n8n board refresh 2026-06-08T17:46:43Z
</commit_message>
<xml_diff>
--- a/app/reports/AMTM_research.xlsx
+++ b/app/reports/AMTM_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-07 17:39 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-08 17:39 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.79</v>
+        <v>0.789</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>32.47</v>
+        <v>32.35</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>22.8</v>
+        <v>22.745</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.424</v>
+        <v>0.422</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.924</v>
+        <v>0.922</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04535999774932861</v>
+        <v>0.04552000045776367</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>244316317.1929824</v>
+        <v>244316337.8324907</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>22.8</v>
+        <v>22.745</v>
       </c>
     </row>
     <row r="38">
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>5570412032</v>
+        <v>5556975104</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>38</v>
+        <v>37.91</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>9.18</v>
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>4814003712</v>
+        <v>4768637440</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>19.011906</v>
+        <v>18.832739</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>12.422</v>
@@ -1568,10 +1568,10 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>6073101824</v>
+        <v>6084995584</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>18.354078</v>
+        <v>18.390022</v>
       </c>
       <c r="E7" s="34" t="n">
         <v>17.109</v>
@@ -1592,10 +1592,10 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>6725088256</v>
+        <v>6638723584</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>59.04636</v>
+        <v>58.28808</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>22.229</v>
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>4508651008</v>
+        <v>4443987968</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>10.4896755</v>
+        <v>10.339232</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>10.6</v>
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>11667101696</v>
+        <v>11761198080</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>41.657238</v>
+        <v>41.993214</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>22.597</v>
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>6680655872</v>
+        <v>6604761088</v>
       </c>
       <c r="D11" s="34" t="n"/>
       <c r="E11" s="34" t="n">
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>6735017472</v>
+        <v>6801058304</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-09T17:48:23Z
</commit_message>
<xml_diff>
--- a/app/reports/AMTM_research.xlsx
+++ b/app/reports/AMTM_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-08 17:39 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-09 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.789</v>
+        <v>0.805</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>32.35</v>
+        <v>32.5</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>22.745</v>
+        <v>22.23</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.422</v>
+        <v>0.462</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.922</v>
+        <v>0.962</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04552000045776367</v>
+        <v>0.04532000064849853</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>244316337.8324907</v>
+        <v>244316312.0107962</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>22.745</v>
+        <v>22.23</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>5556975104</v>
+        <v>5431151616</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>37.91</v>
+        <v>37.05</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>9.18</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>4768637440</v>
+        <v>4817168896</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>18.832739</v>
+        <v>19.04708</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>12.422</v>
+        <v>12.355</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.428</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>6084995584</v>
+        <v>6194699264</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>18.390022</v>
+        <v>18.7015</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>17.109</v>
+        <v>17.151</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>9.907</v>
+        <v>9.932</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>6638723584</v>
+        <v>6835965440</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>58.28808</v>
+        <v>60.019867</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>22.229</v>
+        <v>22.236</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>3.955</v>
+        <v>3.957</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>4443987968</v>
+        <v>4465542656</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>10.339232</v>
+        <v>10.38938</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>10.6</v>
+        <v>10.533</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.901</v>
+        <v>0.896</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>11761198080</v>
+        <v>11832642560</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>41.993214</v>
+        <v>42.152935</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>22.597</v>
+        <v>22.82</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.073</v>
+        <v>3.103</v>
       </c>
     </row>
     <row r="11">
@@ -1664,14 +1664,14 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>6604761088</v>
+        <v>6317754368</v>
       </c>
       <c r="D11" s="34" t="n"/>
       <c r="E11" s="34" t="n">
-        <v>73.134</v>
+        <v>72.92700000000001</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>7.245</v>
+        <v>7.225</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>6801058304</v>
+        <v>6993572352</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>20.72</v>
+        <v>20.979</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>3.626</v>
+        <v>3.672</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-10T17:47:40Z
</commit_message>
<xml_diff>
--- a/app/reports/AMTM_research.xlsx
+++ b/app/reports/AMTM_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-09 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-10 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.805</v>
+        <v>0.802</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>32.5</v>
+        <v>32.38</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>22.23</v>
+        <v>22.25</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.462</v>
+        <v>0.455</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.962</v>
+        <v>0.955</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04532000064849853</v>
+        <v>0.04547999858856201</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>244316312.0107962</v>
+        <v>244316321.0786517</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>22.23</v>
+        <v>22.25</v>
       </c>
     </row>
     <row r="38">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>5431151616</v>
+        <v>5436038144</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>37.05</v>
+        <v>37.08</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>9.130000000000001</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>0.64</v>
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>4817168896</v>
+        <v>4899010048</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>19.04708</v>
+        <v>19.34762</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>12.355</v>
+        <v>12.436</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.42</v>
+        <v>1.429</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>6194699264</v>
+        <v>6129551360</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>18.7015</v>
+        <v>18.544575</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>17.151</v>
+        <v>17.238</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>9.932</v>
+        <v>9.981999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>6835965440</v>
+        <v>6955698688</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>60.019867</v>
+        <v>61.071125</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>22.236</v>
+        <v>23.082</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>3.957</v>
+        <v>4.107</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>4465542656</v>
+        <v>4380593152</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>10.38938</v>
+        <v>10.19174</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>10.533</v>
+        <v>10.554</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.896</v>
+        <v>0.897</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>11832642560</v>
+        <v>12412592128</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>42.152935</v>
+        <v>44.218964</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>22.82</v>
+        <v>23.545</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.103</v>
+        <v>3.202</v>
       </c>
     </row>
     <row r="11">
@@ -1664,14 +1664,14 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>6317754368</v>
+        <v>6493080576</v>
       </c>
       <c r="D11" s="34" t="n"/>
       <c r="E11" s="34" t="n">
-        <v>72.92700000000001</v>
+        <v>71.598</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>7.225</v>
+        <v>7.093</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>6993572352</v>
+        <v>7007014912</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>20.979</v>
+        <v>21.814</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>3.672</v>
+        <v>3.818</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-11T17:47:33Z
</commit_message>
<xml_diff>
--- a/app/reports/AMTM_research.xlsx
+++ b/app/reports/AMTM_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-10 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-11 17:40 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.802</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>32.38</v>
+        <v>32.53</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>22.25</v>
+        <v>21.995</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.455</v>
+        <v>0.479</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.955</v>
+        <v>0.979</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04547999858856201</v>
+        <v>0.04527999877929687</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>244316321.0786517</v>
+        <v>244316320.6183223</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>22.25</v>
+        <v>21.995</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>5436038144</v>
+        <v>5373737472</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>37.08</v>
+        <v>36.66</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>9.109999999999999</v>
+        <v>8.99</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>4899010048</v>
+        <v>4767582208</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>19.34762</v>
+        <v>18.828573</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>12.436</v>
+        <v>12.418</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.429</v>
+        <v>1.427</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>6129551360</v>
+        <v>6075945984</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>18.544575</v>
+        <v>18.362673</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>17.238</v>
+        <v>17.13</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>9.981999999999999</v>
+        <v>9.919</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>6955698688</v>
+        <v>7282117120</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>61.071125</v>
+        <v>63.937084</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>23.082</v>
+        <v>22.756</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>4.107</v>
+        <v>4.049</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>4380593152</v>
+        <v>4419365376</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>10.19174</v>
+        <v>10.281947</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>10.554</v>
+        <v>10.341</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.897</v>
+        <v>0.879</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>12412592128</v>
+        <v>12597142528</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>44.218964</v>
+        <v>44.82582</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>23.545</v>
+        <v>23.372</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.202</v>
+        <v>3.178</v>
       </c>
     </row>
     <row r="11">
@@ -1664,14 +1664,14 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>6493080576</v>
+        <v>6932597760</v>
       </c>
       <c r="D11" s="34" t="n"/>
       <c r="E11" s="34" t="n">
-        <v>71.598</v>
+        <v>70.33799999999999</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>7.093</v>
+        <v>6.968</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>7007014912</v>
+        <v>7230322176</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>21.814</v>
+        <v>21.407</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>3.818</v>
+        <v>3.746</v>
       </c>
     </row>
     <row r="13">

</xml_diff>